<commit_message>
Adapted execution scripts and evaluation logs
</commit_message>
<xml_diff>
--- a/results/result_evaluation_logs/A_Initial_Baseline_Baseline.xlsx
+++ b/results/result_evaluation_logs/A_Initial_Baseline_Baseline.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X51"/>
+  <dimension ref="A1:W51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,11 +544,6 @@
           <t>Result String</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Langfuse Trace ID</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -619,12 +614,10 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q25095540;P31;Q11329&lt;/relation&gt;\n&lt;relation&gt;Q25095540;P175;Q364841&lt;/relation&gt;\n&lt;relation&gt;Q25095540;P264;Q1516254&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 61, 'prompt_tokens': 2686, 'total_tokens': 2747, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-9c562cbb50d946118c43cffc11aa47f3', 'finish_reason': 'stop', 'logprobs': None} id='run-fd86c7be-c921-424e-8954-440f8e13b176-0' usage_metadata={'input_tokens': 2686, 'output_tokens': 61, 'total_tokens': 2747, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>603b5f13-a095-496a-914f-ca557e71efff</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q25095540&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q11329&gt; .
+&lt;http://www.wikidata.org/entity/Q25095540&gt; wd:P175 &lt;http://www.wikidata.org/entity/Q364841&gt; .
+&lt;http://www.wikidata.org/entity/Q25095540&gt; wd:P264 &lt;http://www.wikidata.org/entity/Q1516254&gt; .</t>
         </is>
       </c>
     </row>
@@ -697,12 +690,10 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>content='&lt;instruction&gt;Q20992419, Q17516, Q120&lt;/instruction&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;\n&lt;relation&gt;Q20992419;P31;Q20992419&lt;/relation&gt;\n&lt;relation&gt;Q20992419;P1344;Q17516&lt;/relation&gt;\n&lt;relation&gt;Q20992419;P585;Q120&lt;/relation&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 78, 'prompt_tokens': 1966, 'total_tokens': 2044, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-64dae29c410a4326955ab6fc50b145ff', 'finish_reason': 'stop', 'logprobs': None} id='run-9cb31765-2d26-43ef-b1f8-6a8307518ca4-0' usage_metadata={'input_tokens': 1966, 'output_tokens': 78, 'total_tokens': 2044, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>2372c395-00a7-419a-9c7b-c9b32447d05e</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q20992419&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q20992419&gt; .
+&lt;http://www.wikidata.org/entity/Q20992419&gt; wd:P1344 &lt;http://www.wikidata.org/entity/Q17516&gt; .
+&lt;http://www.wikidata.org/entity/Q20992419&gt; wd:P585 &lt;http://www.wikidata.org/entity/Q120&gt; .</t>
         </is>
       </c>
     </row>
@@ -775,12 +766,14 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q466774;P106;Q395&lt;/relation&gt;\n&lt;relation&gt;Q466774;P27;Q142&lt;/relation&gt;\n&lt;relation&gt;Q466774;P108;Q273626&lt;/relation&gt;\n&lt;relation&gt;Q466774;P184;Q370496&lt;/relation&gt;\n&lt;relation&gt;Q273626;P131;Q142&lt;/relation&gt;\n&lt;relation&gt;Q632552;P397;Q142&lt;/relation&gt;\n&lt;relation&gt;Q370496;P184;Q466774&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 117, 'prompt_tokens': 2351, 'total_tokens': 2468, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-c004133cf52547048004519db354f84d', 'finish_reason': 'stop', 'logprobs': None} id='run-2ee765fa-4324-4758-89a1-29a4e240e530-0' usage_metadata={'input_tokens': 2351, 'output_tokens': 117, 'total_tokens': 2468, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>a32e4e04-c46c-4d8f-ac01-a79f3fa22e11</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q466774&gt; wd:P106 &lt;http://www.wikidata.org/entity/Q395&gt; .
+&lt;http://www.wikidata.org/entity/Q466774&gt; wd:P27 &lt;http://www.wikidata.org/entity/Q142&gt; .
+&lt;http://www.wikidata.org/entity/Q466774&gt; wd:P108 &lt;http://www.wikidata.org/entity/Q273626&gt; .
+&lt;http://www.wikidata.org/entity/Q466774&gt; wd:P184 &lt;http://www.wikidata.org/entity/Q370496&gt; .
+&lt;http://www.wikidata.org/entity/Q273626&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q142&gt; .
+&lt;http://www.wikidata.org/entity/Q632552&gt; wd:P397 &lt;http://www.wikidata.org/entity/Q142&gt; .
+&lt;http://www.wikidata.org/entity/Q370496&gt; wd:P184 &lt;http://www.wikidata.org/entity/Q466774&gt; .</t>
         </is>
       </c>
     </row>
@@ -828,10 +821,10 @@
         <v>3</v>
       </c>
       <c r="O5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q5" t="n">
         <v>7</v>
@@ -853,12 +846,14 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q72697912;P31;Q11424&lt;/relation&gt;\n&lt;relation&gt;Q72697912;P361;Q1993848&lt;/relation&gt;\n&lt;relation&gt;Q72697912;P8370;Q4557532&lt;/relation&gt;\n&lt;relation&gt;Q72697912;P400;Q723685&lt;/relation&gt;\n&lt;relation&gt;Q81725;P31;Q727019&lt;/relation&gt;\n&lt;relation&gt;Q81725;P131;Q258&lt;/relation&gt;\n&lt;relation&gt;Q258;P150;Q81725&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 126, 'prompt_tokens': 4206, 'total_tokens': 4332, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-ed596529e4e54eb5bf182a43b85a0d91', 'finish_reason': 'stop', 'logprobs': None} id='run-648799f1-20a9-4b13-acef-f42d5c5e168d-0' usage_metadata={'input_tokens': 4206, 'output_tokens': 126, 'total_tokens': 4332, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>70172237-2513-4556-8550-ac8de6f4a0fb</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q72697912&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q11424&gt; .
+&lt;http://www.wikidata.org/entity/Q72697912&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q1993848&gt; .
+&lt;http://www.wikidata.org/entity/Q72697912&gt; wd:P8370 &lt;http://www.wikidata.org/entity/Q4557532&gt; .
+&lt;http://www.wikidata.org/entity/Q72697912&gt; wd:P400 &lt;http://www.wikidata.org/entity/Q723685&gt; .
+&lt;http://www.wikidata.org/entity/Q81725&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q727019&gt; .
+&lt;http://www.wikidata.org/entity/Q81725&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q258&gt; .
+&lt;http://www.wikidata.org/entity/Q258&gt; wd:P150 &lt;http://www.wikidata.org/entity/Q81725&gt; .</t>
         </is>
       </c>
     </row>
@@ -931,12 +926,8 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>content='&lt;instruction&gt;Q36771, Q29999, P27&lt;/instruction&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;\n&lt;relation&gt;Q36771;P27;Q29999&lt;/relation&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 41, 'prompt_tokens': 2018, 'total_tokens': 2059, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-2e4a3c6df9d4434eadc07c4e67f327a4', 'finish_reason': 'stop', 'logprobs': None} id='run-ed06ee58-1bd5-4e3d-a11c-bb42f02a0623-0' usage_metadata={'input_tokens': 2018, 'output_tokens': 41, 'total_tokens': 2059, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>a287159a-cb41-4252-8631-d0cefc1a11a0</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q36771&gt; wd:P27 &lt;http://www.wikidata.org/entity/Q29999&gt; .</t>
         </is>
       </c>
     </row>
@@ -954,7 +945,7 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -963,7 +954,7 @@
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -972,7 +963,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -993,7 +984,7 @@
         <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
         <v>0</v>
@@ -1002,32 +993,16 @@
         <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V7" t="n">
         <v>0</v>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
+          <t>Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
 Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q506252 wd:http://www.wikidata.org'..."
-Traceback:
-Traceback (most recent call last):
-  File "/home/mlautenb/CIExMAS/./results/01_Initial Baseline/agent_system.py", line 176, in &lt;module&gt;
-    score = calculate_scores_from_array(evaluate_doc(turtle_string=turtle_string, doc_id=doc_id,
-                                        ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
-  File "/home/mlautenb/CIExMAS/helper_tools/evaluation.py", line 168, in evaluate_doc
-    raise ValueError(f"Error parsing turtle string: {error}")
-ValueError: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
-Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q506252 wd:http://www.wikidata.org'..."
-</t>
-        </is>
-      </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>28855223-69dc-4e30-b1b1-1b2f7b355753</t>
+"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q506252 wd:http://www.wikidata.org'..."</t>
         </is>
       </c>
     </row>
@@ -1100,12 +1075,10 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>content='&lt;goto&gt;FINISH&lt;/goto&gt;\n&lt;relation&gt;Q2226643;P31;Q65943&lt;/relation&gt;\n&lt;relation&gt;Q2226643;P138;Q28937&lt;/relation&gt;\n&lt;relation&gt;Q2226643;P361;Q1057037&lt;/relation&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 61, 'prompt_tokens': 2738, 'total_tokens': 2799, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-0a9bac4b254e431584519c140ebb95ba', 'finish_reason': 'stop', 'logprobs': None} id='run-65509b45-bbd1-4c48-8be4-cecd2f7d8542-0' usage_metadata={'input_tokens': 2738, 'output_tokens': 61, 'total_tokens': 2799, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>a6744423-2de6-4a23-9c21-0ecd202fc221</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q2226643&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q65943&gt; .
+&lt;http://www.wikidata.org/entity/Q2226643&gt; wd:P138 &lt;http://www.wikidata.org/entity/Q28937&gt; .
+&lt;http://www.wikidata.org/entity/Q2226643&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q1057037&gt; .</t>
         </is>
       </c>
     </row>
@@ -1178,12 +1151,14 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q2601034;P31;Q482994&lt;/relation&gt;\n&lt;relation&gt;Q2601034;P264;Q3939773&lt;/relation&gt;\n&lt;relation&gt;Q2601034;P162;Q2808&lt;/relation&gt;\n&lt;relation&gt;Q2601034;P162;Q2338060&lt;/relation&gt;\n&lt;relation&gt;Q2808;P106;Q639669&lt;/relation&gt;\n&lt;relation&gt;Q2338060;P106;Q48287&lt;/relation&gt;\n&lt;relation&gt;Q2601034;P136;Q11399&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 129, 'prompt_tokens': 3467, 'total_tokens': 3596, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-3caf02b16db44a4ca979d12612efd1f2', 'finish_reason': 'stop', 'logprobs': None} id='run-3dcd6f77-bc4d-4c87-bb13-b790eae5a414-0' usage_metadata={'input_tokens': 3467, 'output_tokens': 129, 'total_tokens': 3596, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X9" t="inlineStr">
-        <is>
-          <t>b51b62ba-d8f7-4bbd-a96c-c7e3c3230044</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q2601034&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q482994&gt; .
+&lt;http://www.wikidata.org/entity/Q2601034&gt; wd:P264 &lt;http://www.wikidata.org/entity/Q3939773&gt; .
+&lt;http://www.wikidata.org/entity/Q2601034&gt; wd:P162 &lt;http://www.wikidata.org/entity/Q2808&gt; .
+&lt;http://www.wikidata.org/entity/Q2601034&gt; wd:P162 &lt;http://www.wikidata.org/entity/Q2338060&gt; .
+&lt;http://www.wikidata.org/entity/Q2808&gt; wd:P106 &lt;http://www.wikidata.org/entity/Q639669&gt; .
+&lt;http://www.wikidata.org/entity/Q2338060&gt; wd:P106 &lt;http://www.wikidata.org/entity/Q48287&gt; .
+&lt;http://www.wikidata.org/entity/Q2601034&gt; wd:P136 &lt;http://www.wikidata.org/entity/Q11399&gt; .</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1176,7 @@
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -1210,7 +1185,7 @@
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
@@ -1219,7 +1194,7 @@
         <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -1240,7 +1215,7 @@
         <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="S10" t="n">
         <v>0</v>
@@ -1249,32 +1224,16 @@
         <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="V10" t="n">
         <v>0</v>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
+          <t>Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
 Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q6782514 wd:http://www.wikidata.or'..."
-Traceback:
-Traceback (most recent call last):
-  File "/home/mlautenb/CIExMAS/./results/01_Initial Baseline/agent_system.py", line 176, in &lt;module&gt;
-    score = calculate_scores_from_array(evaluate_doc(turtle_string=turtle_string, doc_id=doc_id,
-                                        ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
-  File "/home/mlautenb/CIExMAS/helper_tools/evaluation.py", line 168, in evaluate_doc
-    raise ValueError(f"Error parsing turtle string: {error}")
-ValueError: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
-Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q6782514 wd:http://www.wikidata.or'..."
-</t>
-        </is>
-      </c>
-      <c r="X10" t="inlineStr">
-        <is>
-          <t>3da23215-cade-46d3-9366-d3d20ac7bcfc</t>
+"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q6782514 wd:http://www.wikidata.or'..."</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1251,7 @@
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -1301,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
@@ -1310,7 +1269,7 @@
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -1331,7 +1290,7 @@
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="S11" t="n">
         <v>0</v>
@@ -1340,32 +1299,16 @@
         <v>0</v>
       </c>
       <c r="U11" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="V11" t="n">
         <v>0</v>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
+          <t>Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
 Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q85563 wd:http://www.wikidata.org/'..."
-Traceback:
-Traceback (most recent call last):
-  File "/home/mlautenb/CIExMAS/./results/01_Initial Baseline/agent_system.py", line 176, in &lt;module&gt;
-    score = calculate_scores_from_array(evaluate_doc(turtle_string=turtle_string, doc_id=doc_id,
-                                        ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
-  File "/home/mlautenb/CIExMAS/helper_tools/evaluation.py", line 168, in evaluate_doc
-    raise ValueError(f"Error parsing turtle string: {error}")
-ValueError: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
-Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q85563 wd:http://www.wikidata.org/'..."
-</t>
-        </is>
-      </c>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t>5b3d3643-53d7-41de-bf50-a0a768f11dc3</t>
+"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q85563 wd:http://www.wikidata.org/'..."</t>
         </is>
       </c>
     </row>
@@ -1438,12 +1381,11 @@
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q5395743;P31;Q41298&lt;/relation&gt;\n&lt;relation&gt;Q5395743;P921;Q735&lt;/relation&gt;\n&lt;relation&gt;Q5395743;P407;Q1321&lt;/relation&gt;\n&lt;relation&gt;Q5395743;P361;Q806208&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 76, 'prompt_tokens': 3704, 'total_tokens': 3780, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-449fed3f406147f4ab8feeb3f9071ab5', 'finish_reason': 'stop', 'logprobs': None} id='run-cb811f47-302b-4a9f-9c16-65e607717a9f-0' usage_metadata={'input_tokens': 3704, 'output_tokens': 76, 'total_tokens': 3780, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X12" t="inlineStr">
-        <is>
-          <t>a753426f-a27a-45c3-a9d7-82cd2b391380</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q5395743&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q41298&gt; .
+&lt;http://www.wikidata.org/entity/Q5395743&gt; wd:P921 &lt;http://www.wikidata.org/entity/Q735&gt; .
+&lt;http://www.wikidata.org/entity/Q5395743&gt; wd:P407 &lt;http://www.wikidata.org/entity/Q1321&gt; .
+&lt;http://www.wikidata.org/entity/Q5395743&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q806208&gt; .</t>
         </is>
       </c>
     </row>
@@ -1461,7 +1403,7 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
@@ -1470,7 +1412,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -1479,7 +1421,7 @@
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
@@ -1500,7 +1442,7 @@
         <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S13" t="n">
         <v>0</v>
@@ -1509,32 +1451,16 @@
         <v>0</v>
       </c>
       <c r="U13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="V13" t="n">
         <v>0</v>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
+          <t>Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
 Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q516760 wd:http://www.wikidata.org'..."
-Traceback:
-Traceback (most recent call last):
-  File "/home/mlautenb/CIExMAS/./results/01_Initial Baseline/agent_system.py", line 176, in &lt;module&gt;
-    score = calculate_scores_from_array(evaluate_doc(turtle_string=turtle_string, doc_id=doc_id,
-                                        ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
-  File "/home/mlautenb/CIExMAS/helper_tools/evaluation.py", line 168, in evaluate_doc
-    raise ValueError(f"Error parsing turtle string: {error}")
-ValueError: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
-Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q516760 wd:http://www.wikidata.org'..."
-</t>
-        </is>
-      </c>
-      <c r="X13" t="inlineStr">
-        <is>
-          <t>04365d62-5361-493d-be9b-edbc4f889f41</t>
+"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q516760 wd:http://www.wikidata.org'..."</t>
         </is>
       </c>
     </row>
@@ -1552,7 +1478,7 @@
         <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -1561,7 +1487,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -1570,7 +1496,7 @@
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -1591,7 +1517,7 @@
         <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S14" t="n">
         <v>0</v>
@@ -1600,32 +1526,16 @@
         <v>0</v>
       </c>
       <c r="U14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="V14" t="n">
         <v>0</v>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
+          <t>Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
 Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q3561541 wd:http://www.wikidata.or'..."
-Traceback:
-Traceback (most recent call last):
-  File "/home/mlautenb/CIExMAS/./results/01_Initial Baseline/agent_system.py", line 176, in &lt;module&gt;
-    score = calculate_scores_from_array(evaluate_doc(turtle_string=turtle_string, doc_id=doc_id,
-                                        ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
-  File "/home/mlautenb/CIExMAS/helper_tools/evaluation.py", line 168, in evaluate_doc
-    raise ValueError(f"Error parsing turtle string: {error}")
-ValueError: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
-Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q3561541 wd:http://www.wikidata.or'..."
-</t>
-        </is>
-      </c>
-      <c r="X14" t="inlineStr">
-        <is>
-          <t>1f2f560f-965b-4a66-9f45-af09f495a23e</t>
+"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q3561541 wd:http://www.wikidata.or'..."</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1586,7 @@
         <v>3</v>
       </c>
       <c r="P15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q15" t="n">
         <v>6</v>
@@ -1698,12 +1608,15 @@
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q42916999;P361;Q568973&lt;/relation&gt;\n&lt;relation&gt;Q42916999;P155;Q48845659&lt;/relation&gt;\n&lt;relation&gt;Q42916999;P31;Q28221935&lt;/relation&gt;\n&lt;relation&gt;Q42916999;P31;Q794655&lt;/relation&gt;\n&lt;relation&gt;Q42916999;P131;Q1264&lt;/relation&gt;\n&lt;relation&gt;Q568973;P131;Q30&lt;/relation&gt;\n&lt;relation&gt;Q48845659;P131;Q1264&lt;/relation&gt;\n&lt;relation&gt;Q568973;P131;Q30&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 143, 'prompt_tokens': 4551, 'total_tokens': 4694, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-d13a58bcc3b348a7a97124722e6fe9f1', 'finish_reason': 'stop', 'logprobs': None} id='run-ae56eda1-b30e-45b2-96ff-28675de4bc37-0' usage_metadata={'input_tokens': 4551, 'output_tokens': 143, 'total_tokens': 4694, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>5f7391f5-7e12-43aa-a7f6-8dbdaf42145c</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q42916999&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q568973&gt; .
+&lt;http://www.wikidata.org/entity/Q42916999&gt; wd:P155 &lt;http://www.wikidata.org/entity/Q48845659&gt; .
+&lt;http://www.wikidata.org/entity/Q42916999&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q28221935&gt; .
+&lt;http://www.wikidata.org/entity/Q42916999&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q794655&gt; .
+&lt;http://www.wikidata.org/entity/Q42916999&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q1264&gt; .
+&lt;http://www.wikidata.org/entity/Q568973&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q30&gt; .
+&lt;http://www.wikidata.org/entity/Q48845659&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q1264&gt; .
+&lt;http://www.wikidata.org/entity/Q568973&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q30&gt; .</t>
         </is>
       </c>
     </row>
@@ -1751,10 +1664,10 @@
         <v>1</v>
       </c>
       <c r="O16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q16" t="n">
         <v>2</v>
@@ -1776,12 +1689,9 @@
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q3311362;P131;Q66117&lt;/relation&gt;\n&lt;relation&gt;Q3311362;P361;Q96&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 42, 'prompt_tokens': 2096, 'total_tokens': 2138, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-b631e7e8d72b4aa5977201e3c676e2aa', 'finish_reason': 'stop', 'logprobs': None} id='run-bcc9190f-d2a7-4840-8e2f-92f5805a02d6-0' usage_metadata={'input_tokens': 2096, 'output_tokens': 42, 'total_tokens': 2138, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X16" t="inlineStr">
-        <is>
-          <t>301fd72a-df6c-43e1-92fe-6640c384ff9e</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q3311362&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q66117&gt; .
+&lt;http://www.wikidata.org/entity/Q3311362&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q96&gt; .</t>
         </is>
       </c>
     </row>
@@ -1854,12 +1764,9 @@
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q7044514;P136;Q46046&lt;/relation&gt;\n&lt;relation&gt;Q7044514;P175;Q234199&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 43, 'prompt_tokens': 3543, 'total_tokens': 3586, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-67792bb5801d4b84abc1ac96c5d0cb4a', 'finish_reason': 'stop', 'logprobs': None} id='run-8cf769f7-9827-4995-88d8-d5a009c84622-0' usage_metadata={'input_tokens': 3543, 'output_tokens': 43, 'total_tokens': 3586, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X17" t="inlineStr">
-        <is>
-          <t>1381780f-1833-493d-b07c-9ece71401bec</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q7044514&gt; wd:P136 &lt;http://www.wikidata.org/entity/Q46046&gt; .
+&lt;http://www.wikidata.org/entity/Q7044514&gt; wd:P175 &lt;http://www.wikidata.org/entity/Q234199&gt; .</t>
         </is>
       </c>
     </row>
@@ -1932,12 +1839,11 @@
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q607380;P5588;Q782&lt;/relation&gt;\n&lt;relation&gt;Q607380;P183;Q664&lt;/relation&gt;\n&lt;relation&gt;Q607380;P703;Q6933370&lt;/relation&gt;\n&lt;relation&gt;Q607380;P31;Q7432&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 73, 'prompt_tokens': 2265, 'total_tokens': 2338, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-289725e6c33a4f3081d1b04ca65671dc', 'finish_reason': 'stop', 'logprobs': None} id='run-a8af3093-3838-4db3-b870-676ddad235db-0' usage_metadata={'input_tokens': 2265, 'output_tokens': 73, 'total_tokens': 2338, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X18" t="inlineStr">
-        <is>
-          <t>da133fbf-41d3-47b1-934d-ac033673f966</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q607380&gt; wd:P5588 &lt;http://www.wikidata.org/entity/Q782&gt; .
+&lt;http://www.wikidata.org/entity/Q607380&gt; wd:P183 &lt;http://www.wikidata.org/entity/Q664&gt; .
+&lt;http://www.wikidata.org/entity/Q607380&gt; wd:P703 &lt;http://www.wikidata.org/entity/Q6933370&gt; .
+&lt;http://www.wikidata.org/entity/Q607380&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q7432&gt; .</t>
         </is>
       </c>
     </row>
@@ -2010,12 +1916,14 @@
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q5686841;P361;Q794&lt;/relation&gt;\n&lt;relation&gt;Q5686841;P1012;Q308864&lt;/relation&gt;\n&lt;relation&gt;Q5686841;P1012;Q928828&lt;/relation&gt;\n&lt;relation&gt;Q308864;P150;Q1282219&lt;/relation&gt;\n&lt;relation&gt;Q308864;P31;Q34770&lt;/relation&gt;\n&lt;relation&gt;Q928828;P31;Q34770&lt;/relation&gt;\n&lt;relation&gt;Q1282219;P31;Q532&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 126, 'prompt_tokens': 2988, 'total_tokens': 3114, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-d64741230d4e4a84bc6544c492680160', 'finish_reason': 'stop', 'logprobs': None} id='run-2c07ab0a-6d0a-4988-82ed-b0000b0984ff-0' usage_metadata={'input_tokens': 2988, 'output_tokens': 126, 'total_tokens': 3114, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X19" t="inlineStr">
-        <is>
-          <t>328ab96e-7414-404e-b11e-836a424ba10e</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q5686841&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q794&gt; .
+&lt;http://www.wikidata.org/entity/Q5686841&gt; wd:P1012 &lt;http://www.wikidata.org/entity/Q308864&gt; .
+&lt;http://www.wikidata.org/entity/Q5686841&gt; wd:P1012 &lt;http://www.wikidata.org/entity/Q928828&gt; .
+&lt;http://www.wikidata.org/entity/Q308864&gt; wd:P150 &lt;http://www.wikidata.org/entity/Q1282219&gt; .
+&lt;http://www.wikidata.org/entity/Q308864&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q34770&gt; .
+&lt;http://www.wikidata.org/entity/Q928828&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q34770&gt; .
+&lt;http://www.wikidata.org/entity/Q1282219&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q532&gt; .</t>
         </is>
       </c>
     </row>
@@ -2088,12 +1996,8 @@
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q20671544;P106;Q27914&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 26, 'prompt_tokens': 2258, 'total_tokens': 2284, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-55af2bba009d4a7487684d979436becd', 'finish_reason': 'stop', 'logprobs': None} id='run-96e1686a-cca0-48d4-a7c5-c708192db0ac-0' usage_metadata={'input_tokens': 2258, 'output_tokens': 26, 'total_tokens': 2284, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X20" t="inlineStr">
-        <is>
-          <t>edde36e3-b71f-4371-956d-899592535258</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q20671544&gt; wd:P106 &lt;http://www.wikidata.org/entity/Q27914&gt; .</t>
         </is>
       </c>
     </row>
@@ -2166,12 +2070,13 @@
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q3048624;P27;Q16&lt;/relation&gt;\n&lt;relation&gt;Q3048624;P141;Q1860&lt;/relation&gt;\n&lt;relation&gt;Q3048624;P106;Q82955&lt;/relation&gt;\n&lt;relation&gt;Q16;Q233492;Q81056&lt;/relation&gt;\n&lt;relation&gt;Q16;P94;Q41549&lt;/relation&gt;\n&lt;relation&gt;Q16;P122;Q41614&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 105, 'prompt_tokens': 4015, 'total_tokens': 4120, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-1360afbb79c14fbf88252dfa24bad809', 'finish_reason': 'stop', 'logprobs': None} id='run-bece48df-ea4b-40de-817e-cd7757e77777-0' usage_metadata={'input_tokens': 4015, 'output_tokens': 105, 'total_tokens': 4120, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X21" t="inlineStr">
-        <is>
-          <t>40458c55-ec72-41f2-bfe5-48a91c4492fc</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q3048624&gt; wd:P27 &lt;http://www.wikidata.org/entity/Q16&gt; .
+&lt;http://www.wikidata.org/entity/Q3048624&gt; wd:P141 &lt;http://www.wikidata.org/entity/Q1860&gt; .
+&lt;http://www.wikidata.org/entity/Q3048624&gt; wd:P106 &lt;http://www.wikidata.org/entity/Q82955&gt; .
+&lt;http://www.wikidata.org/entity/Q16&gt; wd:Q233492 &lt;http://www.wikidata.org/entity/Q81056&gt; .
+&lt;http://www.wikidata.org/entity/Q16&gt; wd:P94 &lt;http://www.wikidata.org/entity/Q41549&gt; .
+&lt;http://www.wikidata.org/entity/Q16&gt; wd:P122 &lt;http://www.wikidata.org/entity/Q41614&gt; .</t>
         </is>
       </c>
     </row>
@@ -2244,12 +2149,10 @@
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q17052475;P279;Q11348&lt;/relation&gt;\n&lt;relation&gt;Q17052475;P361;Q395&lt;/relation&gt;\n&lt;relation&gt;Q11348;P361;Q395&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 57, 'prompt_tokens': 1855, 'total_tokens': 1912, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-33e9f69751a8425282481226192cf289', 'finish_reason': 'stop', 'logprobs': None} id='run-86c38ddc-0f6e-4dd6-9481-f0d534362bfd-0' usage_metadata={'input_tokens': 1855, 'output_tokens': 57, 'total_tokens': 1912, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X22" t="inlineStr">
-        <is>
-          <t>a75af801-5730-43b2-ac66-4ffc5400e66f</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q17052475&gt; wd:P279 &lt;http://www.wikidata.org/entity/Q11348&gt; .
+&lt;http://www.wikidata.org/entity/Q17052475&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q395&gt; .
+&lt;http://www.wikidata.org/entity/Q11348&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q395&gt; .</t>
         </is>
       </c>
     </row>
@@ -2267,7 +2170,7 @@
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
@@ -2276,7 +2179,7 @@
         <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
@@ -2285,7 +2188,7 @@
         <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L23" t="n">
         <v>0</v>
@@ -2306,7 +2209,7 @@
         <v>0</v>
       </c>
       <c r="R23" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S23" t="n">
         <v>0</v>
@@ -2315,32 +2218,16 @@
         <v>0</v>
       </c>
       <c r="U23" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V23" t="n">
         <v>0</v>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
+          <t>Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
 Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q18036690 wd:http://www.wikidata.o'..."
-Traceback:
-Traceback (most recent call last):
-  File "/home/mlautenb/CIExMAS/./results/01_Initial Baseline/agent_system.py", line 176, in &lt;module&gt;
-    score = calculate_scores_from_array(evaluate_doc(turtle_string=turtle_string, doc_id=doc_id,
-                                        ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
-  File "/home/mlautenb/CIExMAS/helper_tools/evaluation.py", line 168, in evaluate_doc
-    raise ValueError(f"Error parsing turtle string: {error}")
-ValueError: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
-Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q18036690 wd:http://www.wikidata.o'..."
-</t>
-        </is>
-      </c>
-      <c r="X23" t="inlineStr">
-        <is>
-          <t>29061f70-d4dd-4a42-90bf-94e4c1aa41f2</t>
+"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q18036690 wd:http://www.wikidata.o'..."</t>
         </is>
       </c>
     </row>
@@ -2413,12 +2300,10 @@
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q188197;P1346;Q1856183&lt;/relation&gt;\n&lt;relation&gt;Q188197;P1346;Q674962&lt;/relation&gt;\n&lt;relation&gt;Q188197;P106;Q59370354&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 61, 'prompt_tokens': 2230, 'total_tokens': 2291, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-7e269753b0d3412e8e2c1fe8157d79e3', 'finish_reason': 'stop', 'logprobs': None} id='run-7ba06f27-f10f-4e3a-9f11-1bf4b54370e1-0' usage_metadata={'input_tokens': 2230, 'output_tokens': 61, 'total_tokens': 2291, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X24" t="inlineStr">
-        <is>
-          <t>7e2a8f56-805a-4e35-9403-aecb56e3b2f1</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q188197&gt; wd:P1346 &lt;http://www.wikidata.org/entity/Q1856183&gt; .
+&lt;http://www.wikidata.org/entity/Q188197&gt; wd:P1346 &lt;http://www.wikidata.org/entity/Q674962&gt; .
+&lt;http://www.wikidata.org/entity/Q188197&gt; wd:P106 &lt;http://www.wikidata.org/entity/Q59370354&gt; .</t>
         </is>
       </c>
     </row>
@@ -2491,12 +2376,12 @@
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q5554167;P86;Q16239205&lt;/relation&gt;\n&lt;relation&gt;Q5554167;P750;Q520445&lt;/relation&gt;\n&lt;relation&gt;Q520445;P31;Q6881511&lt;/relation&gt;\n&lt;relation&gt;Q5554167;P162;Q220072&lt;/relation&gt;\n&lt;relation&gt;Q220072;P31;Q290&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 93, 'prompt_tokens': 3710, 'total_tokens': 3803, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-5b0c95149938442da0e6cb5993cb85d4', 'finish_reason': 'stop', 'logprobs': None} id='run-3feeed4a-1441-4e0b-aff6-95c320eb25b6-0' usage_metadata={'input_tokens': 3710, 'output_tokens': 93, 'total_tokens': 3803, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X25" t="inlineStr">
-        <is>
-          <t>5dc312ff-d79e-448a-bd34-6f812edc72ef</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q5554167&gt; wd:P86 &lt;http://www.wikidata.org/entity/Q16239205&gt; .
+&lt;http://www.wikidata.org/entity/Q5554167&gt; wd:P750 &lt;http://www.wikidata.org/entity/Q520445&gt; .
+&lt;http://www.wikidata.org/entity/Q520445&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q6881511&gt; .
+&lt;http://www.wikidata.org/entity/Q5554167&gt; wd:P162 &lt;http://www.wikidata.org/entity/Q220072&gt; .
+&lt;http://www.wikidata.org/entity/Q220072&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q290&gt; .</t>
         </is>
       </c>
     </row>
@@ -2569,12 +2454,16 @@
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q62066211;P861;Q62066735&lt;/relation&gt;\n&lt;relation&gt;Q62066211;P861;Q62066751&lt;/relation&gt;\n&lt;relation&gt;Q62066211;P1119;Q486396&lt;/relation&gt;\n&lt;relation&gt;Q62066211;P1119;Q11244&lt;/relation&gt;\n&lt;relation&gt;Q62066211;P607;Q486296&lt;/relation&gt;\n&lt;relation&gt;Q62066211;P607;Q698752&lt;/relation&gt;\n&lt;relation&gt;Q62066735;P131;Q62066211&lt;/relation&gt;\n&lt;relation&gt;Q62066751;P131;Q62066211&lt;/relation&gt;\n&lt;relation&gt;Q62066211;P131;Q62066211&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 169, 'prompt_tokens': 3875, 'total_tokens': 4044, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-7038fe9c655b406e816a854ecfd38ea4', 'finish_reason': 'stop', 'logprobs': None} id='run-55d81cb1-dd05-4ed9-953c-bea0e86da874-0' usage_metadata={'input_tokens': 3875, 'output_tokens': 169, 'total_tokens': 4044, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X26" t="inlineStr">
-        <is>
-          <t>c91bb5ff-83a2-433c-9393-4cb54369c2c4</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q62066211&gt; wd:P861 &lt;http://www.wikidata.org/entity/Q62066735&gt; .
+&lt;http://www.wikidata.org/entity/Q62066211&gt; wd:P861 &lt;http://www.wikidata.org/entity/Q62066751&gt; .
+&lt;http://www.wikidata.org/entity/Q62066211&gt; wd:P1119 &lt;http://www.wikidata.org/entity/Q486396&gt; .
+&lt;http://www.wikidata.org/entity/Q62066211&gt; wd:P1119 &lt;http://www.wikidata.org/entity/Q11244&gt; .
+&lt;http://www.wikidata.org/entity/Q62066211&gt; wd:P607 &lt;http://www.wikidata.org/entity/Q486296&gt; .
+&lt;http://www.wikidata.org/entity/Q62066211&gt; wd:P607 &lt;http://www.wikidata.org/entity/Q698752&gt; .
+&lt;http://www.wikidata.org/entity/Q62066735&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q62066211&gt; .
+&lt;http://www.wikidata.org/entity/Q62066751&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q62066211&gt; .
+&lt;http://www.wikidata.org/entity/Q62066211&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q62066211&gt; .</t>
         </is>
       </c>
     </row>
@@ -2592,7 +2481,7 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -2601,7 +2490,7 @@
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
@@ -2610,7 +2499,7 @@
         <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
@@ -2631,7 +2520,7 @@
         <v>0</v>
       </c>
       <c r="R27" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="S27" t="n">
         <v>0</v>
@@ -2640,32 +2529,16 @@
         <v>0</v>
       </c>
       <c r="U27" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="V27" t="n">
         <v>0</v>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
+          <t>Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
 Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q2094579 wd:http://www.wikidata.or'..."
-Traceback:
-Traceback (most recent call last):
-  File "/home/mlautenb/CIExMAS/./results/01_Initial Baseline/agent_system.py", line 176, in &lt;module&gt;
-    score = calculate_scores_from_array(evaluate_doc(turtle_string=turtle_string, doc_id=doc_id,
-                                        ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
-  File "/home/mlautenb/CIExMAS/helper_tools/evaluation.py", line 168, in evaluate_doc
-    raise ValueError(f"Error parsing turtle string: {error}")
-ValueError: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
-Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q2094579 wd:http://www.wikidata.or'..."
-</t>
-        </is>
-      </c>
-      <c r="X27" t="inlineStr">
-        <is>
-          <t>7cbef2d7-ad88-4999-aa83-be8c75d6d03e</t>
+"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q2094579 wd:http://www.wikidata.or'..."</t>
         </is>
       </c>
     </row>
@@ -2713,10 +2586,10 @@
         <v>2</v>
       </c>
       <c r="O28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q28" t="n">
         <v>3</v>
@@ -2738,12 +2611,11 @@
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q22082365;P276;Q965&lt;/relation&gt;\n&lt;relation&gt;Q965;P463;Q47543&lt;/relation&gt;\n&lt;relation&gt;Q22082365;P17;Q965&lt;/relation&gt;\n&lt;relation&gt;Q965;P17;Q2&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 70, 'prompt_tokens': 2385, 'total_tokens': 2455, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-e40a4f67bf0442e1b7d1b42086cf64e0', 'finish_reason': 'stop', 'logprobs': None} id='run-2e839b71-08f8-436e-934c-2d33bae24306-0' usage_metadata={'input_tokens': 2385, 'output_tokens': 70, 'total_tokens': 2455, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X28" t="inlineStr">
-        <is>
-          <t>d533dadc-16ff-4b79-8dae-d9725ae7409e</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q22082365&gt; wd:P276 &lt;http://www.wikidata.org/entity/Q965&gt; .
+&lt;http://www.wikidata.org/entity/Q965&gt; wd:P463 &lt;http://www.wikidata.org/entity/Q47543&gt; .
+&lt;http://www.wikidata.org/entity/Q22082365&gt; wd:P17 &lt;http://www.wikidata.org/entity/Q965&gt; .
+&lt;http://www.wikidata.org/entity/Q965&gt; wd:P17 &lt;http://www.wikidata.org/entity/Q2&gt; .</t>
         </is>
       </c>
     </row>
@@ -2816,12 +2688,15 @@
       </c>
       <c r="W29" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q16926803;P361;Q8062829&lt;/relation&gt;\n&lt;relation&gt;Q16926803;P642;Q2060470&lt;/relation&gt;\n&lt;relation&gt;Q16926803;P642;Q2060470&lt;/relation&gt;\n&lt;relation&gt;Q16926803;P642;Q6811747&lt;/relation&gt;\n&lt;relation&gt;Q16926803;P642;Q6762533&lt;/relation&gt;\n&lt;relation&gt;Q8062829;P31;Q335485&lt;/relation&gt;\n&lt;relation&gt;Q2060470;P131;Q6811747&lt;/relation&gt;\n&lt;relation&gt;Q6762533;P131;Q1065&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 151, 'prompt_tokens': 7294, 'total_tokens': 7445, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-93d5dce51ef74549a499719453886620', 'finish_reason': 'stop', 'logprobs': None} id='run-6e1ac048-5c4a-46f5-9a20-7b11e1b2dc03-0' usage_metadata={'input_tokens': 7294, 'output_tokens': 151, 'total_tokens': 7445, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X29" t="inlineStr">
-        <is>
-          <t>f9cdb951-2dab-4682-be5e-4f2de02f37ce</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q16926803&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q8062829&gt; .
+&lt;http://www.wikidata.org/entity/Q16926803&gt; wd:P642 &lt;http://www.wikidata.org/entity/Q2060470&gt; .
+&lt;http://www.wikidata.org/entity/Q16926803&gt; wd:P642 &lt;http://www.wikidata.org/entity/Q2060470&gt; .
+&lt;http://www.wikidata.org/entity/Q16926803&gt; wd:P642 &lt;http://www.wikidata.org/entity/Q6811747&gt; .
+&lt;http://www.wikidata.org/entity/Q16926803&gt; wd:P642 &lt;http://www.wikidata.org/entity/Q6762533&gt; .
+&lt;http://www.wikidata.org/entity/Q8062829&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q335485&gt; .
+&lt;http://www.wikidata.org/entity/Q2060470&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q6811747&gt; .
+&lt;http://www.wikidata.org/entity/Q6762533&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q1065&gt; .</t>
         </is>
       </c>
     </row>
@@ -2894,12 +2769,12 @@
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q8083051;P131;Q1840968&lt;/relation&gt;\n&lt;relation&gt;Q8083051;P131;Q36&lt;/relation&gt;\n&lt;relation&gt;Q8083051;P421;Q6723&lt;/relation&gt;\n&lt;relation&gt;Q8083051;P421;Q6655&lt;/relation&gt;\n&lt;relation&gt;Q8083051;P31;Q532&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 93, 'prompt_tokens': 4072, 'total_tokens': 4165, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-4ba4ae59e1f3491192db47e4144d6525', 'finish_reason': 'stop', 'logprobs': None} id='run-32314619-c5cf-4d26-9e77-f09cc6ce1be0-0' usage_metadata={'input_tokens': 4072, 'output_tokens': 93, 'total_tokens': 4165, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X30" t="inlineStr">
-        <is>
-          <t>8d97831d-08ed-4397-a095-95b671e19b2e</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q8083051&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q1840968&gt; .
+&lt;http://www.wikidata.org/entity/Q8083051&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q36&gt; .
+&lt;http://www.wikidata.org/entity/Q8083051&gt; wd:P421 &lt;http://www.wikidata.org/entity/Q6723&gt; .
+&lt;http://www.wikidata.org/entity/Q8083051&gt; wd:P421 &lt;http://www.wikidata.org/entity/Q6655&gt; .
+&lt;http://www.wikidata.org/entity/Q8083051&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q532&gt; .</t>
         </is>
       </c>
     </row>
@@ -2972,12 +2847,15 @@
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>content='&lt;goto&gt;FINISH&lt;/goto&gt;\n&lt;relation&gt;Q14707624;P131;Q304801&lt;/relation&gt;\n&lt;relation&gt;Q14707624;P131;Q30&lt;/relation&gt;\n&lt;relation&gt;Q14707624;P269;Q304801&lt;/relation&gt;\n&lt;relation&gt;Q14707624;P269;Q60&lt;/relation&gt;\n&lt;relation&gt;Q304801;P131;Q30&lt;/relation&gt;\n&lt;relation&gt;Q304801;P131;Q60&lt;/relation&gt;\n&lt;relation&gt;Q30;P131;Q60&lt;/relation&gt;\n&lt;relation&gt;Q14707624;P102;Q14827724&lt;/relation&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 137, 'prompt_tokens': 3103, 'total_tokens': 3240, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-aaea148f91ea47ba9d28e92ccf702696', 'finish_reason': 'stop', 'logprobs': None} id='run-887c1a11-5743-4300-9148-a39e3adf7068-0' usage_metadata={'input_tokens': 3103, 'output_tokens': 137, 'total_tokens': 3240, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X31" t="inlineStr">
-        <is>
-          <t>1afc2074-4d14-44c9-a676-0cb9dc1aebf3</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q14707624&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q304801&gt; .
+&lt;http://www.wikidata.org/entity/Q14707624&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q30&gt; .
+&lt;http://www.wikidata.org/entity/Q14707624&gt; wd:P269 &lt;http://www.wikidata.org/entity/Q304801&gt; .
+&lt;http://www.wikidata.org/entity/Q14707624&gt; wd:P269 &lt;http://www.wikidata.org/entity/Q60&gt; .
+&lt;http://www.wikidata.org/entity/Q304801&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q30&gt; .
+&lt;http://www.wikidata.org/entity/Q304801&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q60&gt; .
+&lt;http://www.wikidata.org/entity/Q30&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q60&gt; .
+&lt;http://www.wikidata.org/entity/Q14707624&gt; wd:P102 &lt;http://www.wikidata.org/entity/Q14827724&gt; .</t>
         </is>
       </c>
     </row>
@@ -3050,12 +2928,13 @@
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q64876878;P674;Q65090308&lt;/relation&gt;\n&lt;relation&gt;Q64876878;P725;Q262170&lt;/relation&gt;\n&lt;relation&gt;Q262170;P725;Q64876878&lt;/relation&gt;\n&lt;relation&gt;Q64876878;P527;Q65090308&lt;/relation&gt;\n&lt;relation&gt;Q65090308;P527;Q64876878&lt;/relation&gt;\n&lt;relation&gt;Q262170;P106;Q339616&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 113, 'prompt_tokens': 3218, 'total_tokens': 3331, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-dec6cf6159604d949d258947dabdb3d0', 'finish_reason': 'stop', 'logprobs': None} id='run-471c8e8f-e42a-4010-983f-8983aa520491-0' usage_metadata={'input_tokens': 3218, 'output_tokens': 113, 'total_tokens': 3331, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X32" t="inlineStr">
-        <is>
-          <t>c48b334f-3422-438d-9724-8ec87db60d07</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q64876878&gt; wd:P674 &lt;http://www.wikidata.org/entity/Q65090308&gt; .
+&lt;http://www.wikidata.org/entity/Q64876878&gt; wd:P725 &lt;http://www.wikidata.org/entity/Q262170&gt; .
+&lt;http://www.wikidata.org/entity/Q262170&gt; wd:P725 &lt;http://www.wikidata.org/entity/Q64876878&gt; .
+&lt;http://www.wikidata.org/entity/Q64876878&gt; wd:P527 &lt;http://www.wikidata.org/entity/Q65090308&gt; .
+&lt;http://www.wikidata.org/entity/Q65090308&gt; wd:P527 &lt;http://www.wikidata.org/entity/Q64876878&gt; .
+&lt;http://www.wikidata.org/entity/Q262170&gt; wd:P106 &lt;http://www.wikidata.org/entity/Q339616&gt; .</t>
         </is>
       </c>
     </row>
@@ -3103,10 +2982,10 @@
         <v>3</v>
       </c>
       <c r="O33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q33" t="n">
         <v>5</v>
@@ -3128,12 +3007,16 @@
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q1240173;P131;Q1088790&lt;/relation&gt;\n&lt;relation&gt;Q1240173;P149;Q46261&lt;/relation&gt;\n&lt;relation&gt;Q46261;P361;Q2722661&lt;/relation&gt;\n&lt;relation&gt;Q46261;P361;Q202763&lt;/relation&gt;\n&lt;relation&gt;Q190518;P131;Q28&lt;/relation&gt;\n&lt;relation&gt;Q1088790;P131;Q28&lt;/relation&gt;\n&lt;relation&gt;Q1240173;P149;Q46261&lt;/relation&gt;\n&lt;relation&gt;Q46261;P149;Q2722661&lt;/relation&gt;\n&lt;relation&gt;Q1240173;P585;Q202763&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 159, 'prompt_tokens': 2753, 'total_tokens': 2912, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-1b28fafe0e9b4a0d9c1cfb876425a219', 'finish_reason': 'stop', 'logprobs': None} id='run-aee154fa-4222-48c5-bc95-addc56fda1c2-0' usage_metadata={'input_tokens': 2753, 'output_tokens': 159, 'total_tokens': 2912, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X33" t="inlineStr">
-        <is>
-          <t>5563d935-0953-4da2-ba0a-fa3021fc5e71</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q1240173&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q1088790&gt; .
+&lt;http://www.wikidata.org/entity/Q1240173&gt; wd:P149 &lt;http://www.wikidata.org/entity/Q46261&gt; .
+&lt;http://www.wikidata.org/entity/Q46261&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q2722661&gt; .
+&lt;http://www.wikidata.org/entity/Q46261&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q202763&gt; .
+&lt;http://www.wikidata.org/entity/Q190518&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q28&gt; .
+&lt;http://www.wikidata.org/entity/Q1088790&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q28&gt; .
+&lt;http://www.wikidata.org/entity/Q1240173&gt; wd:P149 &lt;http://www.wikidata.org/entity/Q46261&gt; .
+&lt;http://www.wikidata.org/entity/Q46261&gt; wd:P149 &lt;http://www.wikidata.org/entity/Q2722661&gt; .
+&lt;http://www.wikidata.org/entity/Q1240173&gt; wd:P585 &lt;http://www.wikidata.org/entity/Q202763&gt; .</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3034,7 @@
         <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
@@ -3160,7 +3043,7 @@
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
         <v>0</v>
@@ -3169,7 +3052,7 @@
         <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L34" t="n">
         <v>0</v>
@@ -3190,7 +3073,7 @@
         <v>0</v>
       </c>
       <c r="R34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S34" t="n">
         <v>0</v>
@@ -3199,32 +3082,16 @@
         <v>0</v>
       </c>
       <c r="U34" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V34" t="n">
         <v>0</v>
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
+          <t>Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
 Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q822946 wd:http://www.wikidata.org'..."
-Traceback:
-Traceback (most recent call last):
-  File "/home/mlautenb/CIExMAS/./results/01_Initial Baseline/agent_system.py", line 176, in &lt;module&gt;
-    score = calculate_scores_from_array(evaluate_doc(turtle_string=turtle_string, doc_id=doc_id,
-                                        ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
-  File "/home/mlautenb/CIExMAS/helper_tools/evaluation.py", line 168, in evaluate_doc
-    raise ValueError(f"Error parsing turtle string: {error}")
-ValueError: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
-Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q822946 wd:http://www.wikidata.org'..."
-</t>
-        </is>
-      </c>
-      <c r="X34" t="inlineStr">
-        <is>
-          <t>beb85c45-d465-4967-99cf-cd6e2c45fd95</t>
+"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q822946 wd:http://www.wikidata.org'..."</t>
         </is>
       </c>
     </row>
@@ -3297,12 +3164,10 @@
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q41792848;P106;Q41792848&lt;/relation&gt;\n&lt;relation&gt;Q41792848;P162;Q5072388&lt;/relation&gt;\n&lt;relation&gt;Q5072388;P527;Q5072388&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 63, 'prompt_tokens': 2016, 'total_tokens': 2079, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-9bf012cb794c4ff482eb5d9ea858c87e', 'finish_reason': 'stop', 'logprobs': None} id='run-3df0a89e-aa51-4793-a3ec-2c027152dd48-0' usage_metadata={'input_tokens': 2016, 'output_tokens': 63, 'total_tokens': 2079, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X35" t="inlineStr">
-        <is>
-          <t>7fd2303a-617c-4462-acd1-e35bbd6cafa1</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q41792848&gt; wd:P106 &lt;http://www.wikidata.org/entity/Q41792848&gt; .
+&lt;http://www.wikidata.org/entity/Q41792848&gt; wd:P162 &lt;http://www.wikidata.org/entity/Q5072388&gt; .
+&lt;http://www.wikidata.org/entity/Q5072388&gt; wd:P527 &lt;http://www.wikidata.org/entity/Q5072388&gt; .</t>
         </is>
       </c>
     </row>
@@ -3375,12 +3240,9 @@
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q1490434;P276;Q183&lt;/relation&gt;\n&lt;relation&gt;Q1490434;P31;Q41298&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 42, 'prompt_tokens': 2647, 'total_tokens': 2689, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-d9f262edf3714e55ad928a73643dd46e', 'finish_reason': 'stop', 'logprobs': None} id='run-f600d8bd-a827-498c-a0e9-88d047323c17-0' usage_metadata={'input_tokens': 2647, 'output_tokens': 42, 'total_tokens': 2689, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X36" t="inlineStr">
-        <is>
-          <t>da0f2919-b7e9-47d4-855b-f1f2f5ffcfdb</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q1490434&gt; wd:P276 &lt;http://www.wikidata.org/entity/Q183&gt; .
+&lt;http://www.wikidata.org/entity/Q1490434&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q41298&gt; .</t>
         </is>
       </c>
     </row>
@@ -3453,12 +3315,10 @@
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q2616869;P136;Q132311&lt;/relation&gt;\n&lt;relation&gt;Q2616869;P1433;Q1126800&lt;/relation&gt;\n&lt;relation&gt;Q2616869;P6216;Q19652&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 63, 'prompt_tokens': 2999, 'total_tokens': 3062, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-f07f08c35cc64945b658257aab190457', 'finish_reason': 'stop', 'logprobs': None} id='run-38272ba5-98ec-428a-a318-a7d24775c85e-0' usage_metadata={'input_tokens': 2999, 'output_tokens': 63, 'total_tokens': 3062, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X37" t="inlineStr">
-        <is>
-          <t>0d8f851f-4581-4108-bf0c-526e6298ec5a</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q2616869&gt; wd:P136 &lt;http://www.wikidata.org/entity/Q132311&gt; .
+&lt;http://www.wikidata.org/entity/Q2616869&gt; wd:P1433 &lt;http://www.wikidata.org/entity/Q1126800&gt; .
+&lt;http://www.wikidata.org/entity/Q2616869&gt; wd:P6216 &lt;http://www.wikidata.org/entity/Q19652&gt; .</t>
         </is>
       </c>
     </row>
@@ -3531,12 +3391,12 @@
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>content='&lt;instruction&gt;Meall na Teanga, Q6803534, Munro, Q1320721, Northwest Highlands, Q1084560, Inverness-shire, Q1247390, United Kingdom, Q145, is located in, P131&lt;/instruction&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;\n&lt;relation&gt;Q6803534;P131;Q1084560&lt;/relation&gt;\n&lt;relation&gt;Q6803534;P131;Q1247390&lt;/relation&gt;\n&lt;relation&gt;Q6803534;P131;Q145&lt;/relation&gt;\n&lt;relation&gt;Q6803534;P31;Q1320721&lt;/relation&gt;\n&lt;relation&gt;Q6803534;P31;Q41176&lt;/relation&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 152, 'prompt_tokens': 2339, 'total_tokens': 2491, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-026cbfa4b9e34f15a2ea9337e485483c', 'finish_reason': 'stop', 'logprobs': None} id='run-41615b81-5b71-4dde-a1ac-33c06a5abae3-0' usage_metadata={'input_tokens': 2339, 'output_tokens': 152, 'total_tokens': 2491, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X38" t="inlineStr">
-        <is>
-          <t>1a24e0aa-8c29-4d6f-aabf-19cf56af2ef0</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q6803534&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q1084560&gt; .
+&lt;http://www.wikidata.org/entity/Q6803534&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q1247390&gt; .
+&lt;http://www.wikidata.org/entity/Q6803534&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q145&gt; .
+&lt;http://www.wikidata.org/entity/Q6803534&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q1320721&gt; .
+&lt;http://www.wikidata.org/entity/Q6803534&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q41176&gt; .</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3414,7 @@
         <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
@@ -3563,7 +3423,7 @@
         <v>0</v>
       </c>
       <c r="H39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
@@ -3572,7 +3432,7 @@
         <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L39" t="n">
         <v>0</v>
@@ -3593,7 +3453,7 @@
         <v>0</v>
       </c>
       <c r="R39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S39" t="n">
         <v>0</v>
@@ -3602,32 +3462,16 @@
         <v>0</v>
       </c>
       <c r="U39" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="V39" t="n">
         <v>0</v>
       </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
+          <t>Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
 Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q907827 wd:http://www.wikidata.org'..."
-Traceback:
-Traceback (most recent call last):
-  File "/home/mlautenb/CIExMAS/./results/01_Initial Baseline/agent_system.py", line 176, in &lt;module&gt;
-    score = calculate_scores_from_array(evaluate_doc(turtle_string=turtle_string, doc_id=doc_id,
-                                        ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
-  File "/home/mlautenb/CIExMAS/helper_tools/evaluation.py", line 168, in evaluate_doc
-    raise ValueError(f"Error parsing turtle string: {error}")
-ValueError: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
-Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q907827 wd:http://www.wikidata.org'..."
-</t>
-        </is>
-      </c>
-      <c r="X39" t="inlineStr">
-        <is>
-          <t>05703147-71cd-46e3-929b-f0c3dec015bf</t>
+"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q907827 wd:http://www.wikidata.org'..."</t>
         </is>
       </c>
     </row>
@@ -3700,12 +3544,11 @@
       </c>
       <c r="W40" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q1064344;P361;Q1406&lt;/relation&gt;\n&lt;relation&gt;Q1064344;P361;Q1406&lt;/relation&gt;\n&lt;relation&gt;Q1406;P527;Q1064344&lt;/relation&gt;\n&lt;relation&gt;Q1406;P361;Q2283&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 76, 'prompt_tokens': 3107, 'total_tokens': 3183, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-9aa8a9f274df4377b3b6e921b6faa2a9', 'finish_reason': 'stop', 'logprobs': None} id='run-7fae2acc-76b1-40b1-ba2e-20671c641a23-0' usage_metadata={'input_tokens': 3107, 'output_tokens': 76, 'total_tokens': 3183, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X40" t="inlineStr">
-        <is>
-          <t>ceefd60c-f781-4721-a27c-1a6f42534691</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q1064344&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q1406&gt; .
+&lt;http://www.wikidata.org/entity/Q1064344&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q1406&gt; .
+&lt;http://www.wikidata.org/entity/Q1406&gt; wd:P527 &lt;http://www.wikidata.org/entity/Q1064344&gt; .
+&lt;http://www.wikidata.org/entity/Q1406&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q2283&gt; .</t>
         </is>
       </c>
     </row>
@@ -3778,12 +3621,9 @@
       </c>
       <c r="W41" t="inlineStr">
         <is>
-          <t>content='&lt;instruction&gt;Q47554, Q54153, P36, Q1261531&lt;/instruction&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;\n&lt;relation&gt;Q47554;P36;Q54153&lt;/relation&gt;\n&lt;relation&gt;Q47554;P403;Q1261531&lt;/relation&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 63, 'prompt_tokens': 2049, 'total_tokens': 2112, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-d7033efe78d54eee9df0a29064740dc3', 'finish_reason': 'stop', 'logprobs': None} id='run-b9ba9adc-b33e-44c5-bfe3-4f210038cd50-0' usage_metadata={'input_tokens': 2049, 'output_tokens': 63, 'total_tokens': 2112, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X41" t="inlineStr">
-        <is>
-          <t>76b89fb4-d27b-4f2e-a2db-2c56038eb991</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q47554&gt; wd:P36 &lt;http://www.wikidata.org/entity/Q54153&gt; .
+&lt;http://www.wikidata.org/entity/Q47554&gt; wd:P403 &lt;http://www.wikidata.org/entity/Q1261531&gt; .</t>
         </is>
       </c>
     </row>
@@ -3856,12 +3696,16 @@
       </c>
       <c r="W42" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q54322348;P131;Q16568&lt;/relation&gt;\n&lt;relation&gt;Q16568;P36;Q493605&lt;/relation&gt;\n&lt;relation&gt;Q16568;P190;Q12191&lt;/relation&gt;\n&lt;relation&gt;Q16568;P190;Q42622&lt;/relation&gt;\n&lt;relation&gt;Q54322348;P31;Q41176&lt;/relation&gt;\n&lt;relation&gt;Q16568;P31;Q515&lt;/relation&gt;\n&lt;relation&gt;Q493605;P31;Q28527&lt;/relation&gt;\n&lt;relation&gt;Q12191;P31;Q515&lt;/relation&gt;\n&lt;relation&gt;Q42622;P31;Q515&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 152, 'prompt_tokens': 2695, 'total_tokens': 2847, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-1f63397c0daa488db29f73130c7d123e', 'finish_reason': 'stop', 'logprobs': None} id='run-2407a856-ef51-43ba-8243-484b2c128b7b-0' usage_metadata={'input_tokens': 2695, 'output_tokens': 152, 'total_tokens': 2847, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X42" t="inlineStr">
-        <is>
-          <t>41ec8929-f371-481d-9468-e085860f8aad</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q54322348&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q16568&gt; .
+&lt;http://www.wikidata.org/entity/Q16568&gt; wd:P36 &lt;http://www.wikidata.org/entity/Q493605&gt; .
+&lt;http://www.wikidata.org/entity/Q16568&gt; wd:P190 &lt;http://www.wikidata.org/entity/Q12191&gt; .
+&lt;http://www.wikidata.org/entity/Q16568&gt; wd:P190 &lt;http://www.wikidata.org/entity/Q42622&gt; .
+&lt;http://www.wikidata.org/entity/Q54322348&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q41176&gt; .
+&lt;http://www.wikidata.org/entity/Q16568&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q515&gt; .
+&lt;http://www.wikidata.org/entity/Q493605&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q28527&gt; .
+&lt;http://www.wikidata.org/entity/Q12191&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q515&gt; .
+&lt;http://www.wikidata.org/entity/Q42622&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q515&gt; .</t>
         </is>
       </c>
     </row>
@@ -3934,12 +3778,9 @@
       </c>
       <c r="W43" t="inlineStr">
         <is>
-          <t>content='&lt;instruction&gt;Q87412161, Q5, Q95994024, P3373&lt;/instruction&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;\n&lt;relation&gt;Q87412161;P31;Q5&lt;/relation&gt;\n&lt;relation&gt;Q87412161;P3373;Q95994024&lt;/relation&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 66, 'prompt_tokens': 2045, 'total_tokens': 2111, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-ba7ea19c8d294b9985318ded3706c519', 'finish_reason': 'stop', 'logprobs': None} id='run-db599d1b-e171-4861-a74d-9bd366b01a61-0' usage_metadata={'input_tokens': 2045, 'output_tokens': 66, 'total_tokens': 2111, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X43" t="inlineStr">
-        <is>
-          <t>b6251bbc-3b13-472a-8624-87e6bbfae7c5</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q87412161&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q5&gt; .
+&lt;http://www.wikidata.org/entity/Q87412161&gt; wd:P3373 &lt;http://www.wikidata.org/entity/Q95994024&gt; .</t>
         </is>
       </c>
     </row>
@@ -4012,12 +3853,11 @@
       </c>
       <c r="W44" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q29644512;P31;Q1358919&lt;/relation&gt;\n&lt;relation&gt;Q29644512;P1056;Q1358919&lt;/relation&gt;\n&lt;relation&gt;Q29644512;P569;Q152074&lt;/relation&gt;\n&lt;relation&gt;Q152074;P361;Q29644512&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 80, 'prompt_tokens': 3177, 'total_tokens': 3257, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-390759573b8e4a70bf5768fbe0548fb7', 'finish_reason': 'stop', 'logprobs': None} id='run-8d2089a7-a512-4880-ba77-eb52c93cc86a-0' usage_metadata={'input_tokens': 3177, 'output_tokens': 80, 'total_tokens': 3257, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X44" t="inlineStr">
-        <is>
-          <t>af7ca544-c96d-418f-beb3-64a68d34e8d5</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q29644512&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q1358919&gt; .
+&lt;http://www.wikidata.org/entity/Q29644512&gt; wd:P1056 &lt;http://www.wikidata.org/entity/Q1358919&gt; .
+&lt;http://www.wikidata.org/entity/Q29644512&gt; wd:P569 &lt;http://www.wikidata.org/entity/Q152074&gt; .
+&lt;http://www.wikidata.org/entity/Q152074&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q29644512&gt; .</t>
         </is>
       </c>
     </row>
@@ -4065,10 +3905,10 @@
         <v>3</v>
       </c>
       <c r="O45" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P45" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q45" t="n">
         <v>9</v>
@@ -4090,12 +3930,17 @@
       </c>
       <c r="W45" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q5288565;P31;Q7368&lt;/relation&gt;\n&lt;relation&gt;Q5288565;P495;Q258&lt;/relation&gt;\n&lt;relation&gt;Q5288565;P618;Q42329&lt;/relation&gt;\n&lt;relation&gt;Q42329;P1056;Q197204&lt;/relation&gt;\n&lt;relation&gt;Q5288565;P462;Q23444&lt;/relation&gt;\n&lt;relation&gt;Q5288565;P462;Q23445&lt;/relation&gt;\n&lt;relation&gt;Q7368;P131;Q858177&lt;/relation&gt;\n&lt;relation&gt;Q7368;P1056;Q8495&lt;/relation&gt;\n&lt;relation&gt;Q5288565;P279;Q7368&lt;/relation&gt;\n&lt;relation&gt;Q7368;P31;Q5&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 175, 'prompt_tokens': 4173, 'total_tokens': 4348, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-83dd468416904dc2b1184e0f5899dbe2', 'finish_reason': 'stop', 'logprobs': None} id='run-c29285bc-077e-4cc9-9446-92384b5a8c27-0' usage_metadata={'input_tokens': 4173, 'output_tokens': 175, 'total_tokens': 4348, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X45" t="inlineStr">
-        <is>
-          <t>19162a77-ba31-4d93-94f0-c08283c47081</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q5288565&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q7368&gt; .
+&lt;http://www.wikidata.org/entity/Q5288565&gt; wd:P495 &lt;http://www.wikidata.org/entity/Q258&gt; .
+&lt;http://www.wikidata.org/entity/Q5288565&gt; wd:P618 &lt;http://www.wikidata.org/entity/Q42329&gt; .
+&lt;http://www.wikidata.org/entity/Q42329&gt; wd:P1056 &lt;http://www.wikidata.org/entity/Q197204&gt; .
+&lt;http://www.wikidata.org/entity/Q5288565&gt; wd:P462 &lt;http://www.wikidata.org/entity/Q23444&gt; .
+&lt;http://www.wikidata.org/entity/Q5288565&gt; wd:P462 &lt;http://www.wikidata.org/entity/Q23445&gt; .
+&lt;http://www.wikidata.org/entity/Q7368&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q858177&gt; .
+&lt;http://www.wikidata.org/entity/Q7368&gt; wd:P1056 &lt;http://www.wikidata.org/entity/Q8495&gt; .
+&lt;http://www.wikidata.org/entity/Q5288565&gt; wd:P279 &lt;http://www.wikidata.org/entity/Q7368&gt; .
+&lt;http://www.wikidata.org/entity/Q7368&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q5&gt; .</t>
         </is>
       </c>
     </row>
@@ -4168,12 +4013,10 @@
       </c>
       <c r="W46" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q2061122;P162;Q92560&lt;/relation&gt;\n&lt;relation&gt;Q92560;P837;Q734663&lt;/relation&gt;\n&lt;relation&gt;Q92560;P400;Q231302&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 58, 'prompt_tokens': 2092, 'total_tokens': 2150, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-3ededecbe0db4b0abc2b35e30e0320fa', 'finish_reason': 'stop', 'logprobs': None} id='run-641247ed-37b8-44cb-9669-9a864f7e1324-0' usage_metadata={'input_tokens': 2092, 'output_tokens': 58, 'total_tokens': 2150, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X46" t="inlineStr">
-        <is>
-          <t>17da7931-02ca-4215-9e40-cbe2e87d4b67</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q2061122&gt; wd:P162 &lt;http://www.wikidata.org/entity/Q92560&gt; .
+&lt;http://www.wikidata.org/entity/Q92560&gt; wd:P837 &lt;http://www.wikidata.org/entity/Q734663&gt; .
+&lt;http://www.wikidata.org/entity/Q92560&gt; wd:P400 &lt;http://www.wikidata.org/entity/Q231302&gt; .</t>
         </is>
       </c>
     </row>
@@ -4246,12 +4089,10 @@
       </c>
       <c r="W47" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q18036732;P361;Q753805&lt;/relation&gt;\n&lt;relation&gt;Q753805;P31;Q186380&lt;/relation&gt;\n&lt;relation&gt;Q753805;P279;Q186380&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 58, 'prompt_tokens': 1916, 'total_tokens': 1974, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-fc89f7c225044063b6470e3a55f67cde', 'finish_reason': 'stop', 'logprobs': None} id='run-a91f0131-6a98-4af1-b8c7-c8f862a168b9-0' usage_metadata={'input_tokens': 1916, 'output_tokens': 58, 'total_tokens': 1974, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X47" t="inlineStr">
-        <is>
-          <t>489589fd-bb93-48a0-976f-a2ea4da3e247</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q18036732&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q753805&gt; .
+&lt;http://www.wikidata.org/entity/Q753805&gt; wd:P31 &lt;http://www.wikidata.org/entity/Q186380&gt; .
+&lt;http://www.wikidata.org/entity/Q753805&gt; wd:P279 &lt;http://www.wikidata.org/entity/Q186380&gt; .</t>
         </is>
       </c>
     </row>
@@ -4324,12 +4165,10 @@
       </c>
       <c r="W48" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q977911;P47;Q979352&lt;/relation&gt;\n&lt;relation&gt;Q977911;P131;Q112686&lt;/relation&gt;\n&lt;relation&gt;Q979352;P131;Q112686&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 57, 'prompt_tokens': 2457, 'total_tokens': 2514, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-16c8986113584bd0baa2c09e22edfea1', 'finish_reason': 'stop', 'logprobs': None} id='run-3318ad2c-d9f1-40e6-910a-7dc8f82c2927-0' usage_metadata={'input_tokens': 2457, 'output_tokens': 57, 'total_tokens': 2514, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X48" t="inlineStr">
-        <is>
-          <t>5d1330a6-b5d9-4374-acbe-b5d881d4b73c</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q977911&gt; wd:P47 &lt;http://www.wikidata.org/entity/Q979352&gt; .
+&lt;http://www.wikidata.org/entity/Q977911&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q112686&gt; .
+&lt;http://www.wikidata.org/entity/Q979352&gt; wd:P131 &lt;http://www.wikidata.org/entity/Q112686&gt; .</t>
         </is>
       </c>
     </row>
@@ -4402,12 +4241,14 @@
       </c>
       <c r="W49" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q4546576;P155;Q173071&lt;/relation&gt;\n&lt;relation&gt;Q4546576;P541;Q170386&lt;/relation&gt;\n&lt;relation&gt;Q4546576;P156;Q1358726&lt;/relation&gt;\n&lt;relation&gt;Q173071;P361;Q19546&lt;/relation&gt;\n&lt;relation&gt;Q170386;P361;Q19546&lt;/relation&gt;\n&lt;relation&gt;Q173071;P527;Q5&lt;/relation&gt;\n&lt;relation&gt;Q173071;P1343;Q602358&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 125, 'prompt_tokens': 3398, 'total_tokens': 3523, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-bf1122cfceb74d10814d506341b582d4', 'finish_reason': 'stop', 'logprobs': None} id='run-d342fd8a-83dd-49dc-a2b7-f553aae90b71-0' usage_metadata={'input_tokens': 3398, 'output_tokens': 125, 'total_tokens': 3523, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X49" t="inlineStr">
-        <is>
-          <t>7a81a5c6-a930-4b17-b75b-3ee430494012</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q4546576&gt; wd:P155 &lt;http://www.wikidata.org/entity/Q173071&gt; .
+&lt;http://www.wikidata.org/entity/Q4546576&gt; wd:P541 &lt;http://www.wikidata.org/entity/Q170386&gt; .
+&lt;http://www.wikidata.org/entity/Q4546576&gt; wd:P156 &lt;http://www.wikidata.org/entity/Q1358726&gt; .
+&lt;http://www.wikidata.org/entity/Q173071&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q19546&gt; .
+&lt;http://www.wikidata.org/entity/Q170386&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q19546&gt; .
+&lt;http://www.wikidata.org/entity/Q173071&gt; wd:P527 &lt;http://www.wikidata.org/entity/Q5&gt; .
+&lt;http://www.wikidata.org/entity/Q173071&gt; wd:P1343 &lt;http://www.wikidata.org/entity/Q602358&gt; .</t>
         </is>
       </c>
     </row>
@@ -4425,7 +4266,7 @@
         <v>0</v>
       </c>
       <c r="E50" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F50" t="n">
         <v>0</v>
@@ -4434,7 +4275,7 @@
         <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>
@@ -4443,7 +4284,7 @@
         <v>0</v>
       </c>
       <c r="K50" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L50" t="n">
         <v>0</v>
@@ -4464,7 +4305,7 @@
         <v>0</v>
       </c>
       <c r="R50" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S50" t="n">
         <v>0</v>
@@ -4473,32 +4314,16 @@
         <v>0</v>
       </c>
       <c r="U50" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="V50" t="n">
         <v>0</v>
       </c>
       <c r="W50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
+          <t>Error: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
 Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q2822458 wd:http://www.wikidata.or'..."
-Traceback:
-Traceback (most recent call last):
-  File "/home/mlautenb/CIExMAS/./results/01_Initial Baseline/agent_system.py", line 176, in &lt;module&gt;
-    score = calculate_scores_from_array(evaluate_doc(turtle_string=turtle_string, doc_id=doc_id,
-                                        ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
-  File "/home/mlautenb/CIExMAS/helper_tools/evaluation.py", line 168, in evaluate_doc
-    raise ValueError(f"Error parsing turtle string: {error}")
-ValueError: Error parsing turtle string: Error: at line 2 of &lt;&gt;:
-Bad syntax (expected '.' or '}' or ']' at end of statement) at ^ in:
-"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q2822458 wd:http://www.wikidata.or'..."
-</t>
-        </is>
-      </c>
-      <c r="X50" t="inlineStr">
-        <is>
-          <t>d31fac8d-e57d-4c34-b397-2c4d0d9d7846</t>
+"b'@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .\nwd:http:'^b'//www.wikidata.org/entity/Q2822458 wd:http://www.wikidata.or'..."</t>
         </is>
       </c>
     </row>
@@ -4571,12 +4396,8 @@
       </c>
       <c r="W51" t="inlineStr">
         <is>
-          <t>content='&lt;relation&gt;Q2362697;P361;Q503601&lt;/relation&gt;\n&lt;goto&gt;FINISH&lt;/goto&gt;' additional_kwargs={'refusal': None} response_metadata={'token_usage': {'completion_tokens': 26, 'prompt_tokens': 1845, 'total_tokens': 1871, 'completion_tokens_details': None, 'prompt_tokens_details': None}, 'model_name': 'kosbu/Llama-3.3-70B-Instruct-AWQ', 'system_fingerprint': None, 'id': 'chatcmpl-5ace8ccbe6dd4ea9b1b9c964339fce0b', 'finish_reason': 'stop', 'logprobs': None} id='run-30035d4a-5014-4d44-afc2-ac231205d165-0' usage_metadata={'input_tokens': 1845, 'output_tokens': 26, 'total_tokens': 1871, 'input_token_details': {}, 'output_token_details': {}}</t>
-        </is>
-      </c>
-      <c r="X51" t="inlineStr">
-        <is>
-          <t>cb04aa67-b048-4c79-9728-aa5014ed3d0b</t>
+          <t>@prefix wd: &lt;http://www.wikidata.org/entity/&gt; .
+&lt;http://www.wikidata.org/entity/Q2362697&gt; wd:P361 &lt;http://www.wikidata.org/entity/Q503601&gt; .</t>
         </is>
       </c>
     </row>

</xml_diff>